<commit_message>
research(product-scan): re-index scoring on fintech/crypto/AI; confirm COO handling
- Domain fit re-scored to prioritize fintech/crypto/payments (5), AI/ML (4),
  data/infra/dev-tools/security SaaS (3), other vertical incl. health (2), none (1).
  Health weighting removed. Hint map now applies to both Consider and direct-ATS paths.
- COO/Chief Operating Officer stays in the title filter; verified 0 are currently
  posted on these boards (filled via exec search, not public listings).
- Regenerated csv/md/xlsx/pdf. 18 roles (fit 5x6, 4x4, 3x4, 2x3, 1x1); top tier now
  Affirm, Flex, Brex, Tala, Rippling (fintech), then Runlayer/Owner/Instacart (AI).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011C7n5R5VxejCKFAN8WmUQg
</commit_message>
<xml_diff>
--- a/research/fp-a-role-scan/product_leadership_roles.xlsx
+++ b/research/fp-a-role-scan/product_leadership_roles.xlsx
@@ -45,7 +45,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -77,11 +77,6 @@
         <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -109,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -134,9 +129,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -524,7 +516,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Product &amp; exec leadership roles • Director/Head/VP Product · CPO · COO · Founding PM • eligible with 12 yrs (min ≤12) • Remote-US or Dallas–Fort Worth or San Francisco • posted ≤60 days</t>
+          <t>Product &amp; exec leadership • Director/Head/VP Product · CPO · COO · Founding PM • eligible with 12 yrs (min ≤12) • Remote-US / Dallas–Fort Worth / San Francisco • posted ≤60 days • Fit indexed on fintech/crypto/AI (5=fintech/crypto, 4=AI, 3=infra/SaaS, 2=other, 1=none)</t>
         </is>
       </c>
     </row>
@@ -598,22 +590,22 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>IVP, Venrock</t>
+          <t>Craft Ventures, Founders Fund</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Aledade</t>
+          <t>Affirm</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Public (AFRM)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Director of Product Management (Internal AI Product Strategy &amp; Ops), Remote</t>
+          <t>Director of Product Management, Financial Platforms</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -623,7 +615,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>n/s</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -633,13 +625,13 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>payer / health-insurance economics is the core product</t>
+          <t>fintech / crypto / payments — priority domain</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -656,12 +648,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>GV, IVP, Venrock, Lightspeed</t>
+          <t>Lightspeed</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Aledade</t>
+          <t>Flex</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -671,7 +663,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Director of Product Management (Salesforce), Remote</t>
+          <t>Director of Product Management, CS/AI</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -681,147 +673,143 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>San Francisco: San Francisco, California (in-office)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>$210,800–$310,000</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>fintech / crypto / payments — priority domain</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>IVP</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Brex</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product, Growth/AI</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>San Francisco: San Francisco, California, United States</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>fintech / crypto / payments — priority domain</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Tala</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>director</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
           <t>12+</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>$180,000–$285,000</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>payer / health-insurance economics is the core product</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Oak HC/FT, Sequoia</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Maven Clinic</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>VP of Product, Healthcare</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>vp</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10+</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>$200,000–$300,000</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>healthcare / health-tech (non-payer)</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Craft Ventures, Founders Fund</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Affirm</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Public (AFRM)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Director of Product Management, Financial Platforms</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>fintech / payments / insurtech (adjacent domain)</t>
+          <t>fintech / crypto / payments — priority domain</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -831,9 +819,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -853,7 +841,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Director of Product Management, CS/AI</t>
+          <t>Director of Product, Payments Platform</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -863,85 +851,81 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>7+</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>San Francisco: San Francisco, California (in-office)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>$248,000–$310,000</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>fintech / crypto / payments — priority domain</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Founders Fund</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Rippling</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Senior Director of Product Management, Payroll</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
           <t>n/s</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco: San Francisco, California (in-office)</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>$210,800–$310,000</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>fintech / payments / insurtech (adjacent domain)</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>GV</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Tala</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Director of Product</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>director</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>12+</t>
-        </is>
-      </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
+          <t>San Francisco: San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>fintech / payments / insurtech (adjacent domain)</t>
+          <t>fintech / crypto / payments — priority domain</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -951,19 +935,19 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Lightspeed</t>
+          <t>Felicis</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Flex</t>
+          <t>Runlayer</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -973,281 +957,277 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Director of Product, Payments Platform</t>
+          <t>Founding Product Manager, Control Plane</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
+          <t>mid</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>$135,000–$220,000</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Felicis</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Runlayer</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Founding Product Manager, Agents</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>mid</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>$135,000–$220,000</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>IVP, Venrock</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Aledade</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product Management (Internal AI Product Strategy &amp; Ops), Remote</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>GV, Kleiner Perkins</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Motive</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product, Workforce Management</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
           <t>director</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>7+</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco: San Francisco, California (in-office)</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>$248,000–$310,000</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>fintech / payments / insurtech (adjacent domain)</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Felicis</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Runlayer</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>$208,000–$299,000</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Redpoint</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Private</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Founding Product Manager, Control Plane</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>mid</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>n/s</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Founding PM - Reporting &amp; Agentic Insights</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>5+</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>$135,000–$220,000</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>vertical/horizontal SaaS — no domain overlap</t>
-        </is>
-      </c>
-      <c r="L10" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Felicis</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Runlayer</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Founding Product Manager, Agents</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>mid</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>n/s</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>$135,000–$220,000</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>vertical/horizontal SaaS — no domain overlap</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>a16z</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Tanium</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Director of Product Management - Endpoint Management Partner Integrations</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>director</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>8+</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>DFW: DFW (hybrid)</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>$214,000–$328,000</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>vertical/horizontal SaaS — no domain overlap</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>IVP</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Brex</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Director of Product, Growth/AI</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>10+</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco: San Francisco, California, United States</t>
-        </is>
-      </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>vertical/horizontal SaaS — no domain overlap</t>
+          <t>AI / ML — priority domain</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -1257,9 +1237,9 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1309,7 +1289,7 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>vertical/horizontal SaaS — no domain overlap</t>
+          <t>AI / ML — priority domain</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1319,9 +1299,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1371,7 +1351,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>no domain overlap</t>
+          <t>data / infra / dev-tools / security SaaS</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1381,19 +1361,19 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>GV, Kleiner Perkins</t>
+          <t>a16z</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Motive</t>
+          <t>Tanium</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1403,7 +1383,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Director of Product, Workforce Management</t>
+          <t>Director of Product Management - Endpoint Management Partner Integrations</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1413,27 +1393,27 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>10+</t>
+          <t>8+</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Remote (US)</t>
+          <t>DFW: DFW (hybrid)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>$208,000–$299,000</t>
+          <t>$214,000–$328,000</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>no domain overlap</t>
+          <t>data / infra / dev-tools / security SaaS</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1443,9 +1423,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1491,7 +1471,7 @@
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>no domain overlap</t>
+          <t>data / infra / dev-tools / security SaaS</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1501,19 +1481,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Redpoint</t>
+          <t>IVP</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Genlogs</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1523,7 +1503,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Founding PM - Reporting &amp; Agentic Insights</t>
+          <t>Director of Product- Shippers</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1533,7 +1513,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>5+</t>
+          <t>n/s</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1541,15 +1521,11 @@
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
+      <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>no domain overlap</t>
+          <t>data / infra / dev-tools / security SaaS</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1559,19 +1535,19 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Founders Fund</t>
+          <t>Oak HC/FT, Sequoia</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Rippling</t>
+          <t>Maven Clinic</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1581,29 +1557,37 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Senior Director of Product Management, Payroll</t>
+          <t>VP of Product, Healthcare</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>vp</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>n/s</t>
+          <t>10+</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>San Francisco: San Francisco, CA</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr"/>
-      <c r="J19" s="4" t="inlineStr"/>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>$200,000–$300,000</t>
+        </is>
+      </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>no domain overlap</t>
+          <t>other vertical (consumer / health / logistics / etc.)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1613,19 +1597,19 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>IVP</t>
+          <t>GV, IVP, Venrock, Lightspeed</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Genlogs</t>
+          <t>Aledade</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1635,17 +1619,17 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Director of Product- Shippers</t>
+          <t>Director of Product Management (Salesforce), Remote</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>director</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>n/s</t>
+          <t>12+</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1653,11 +1637,19 @@
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>$180,000–$285,000</t>
+        </is>
+      </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>no domain overlap</t>
+          <t>other vertical (consumer / health / logistics / etc.)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">

</xml_diff>

<commit_message>
research(product-scan): expand to any US location; fix location matching
- Per request, broadened location from Remote/DFW/SF to ANY US location (remote-US
  or any US metro; in-office/hybrid OK). Foreign-only roles excluded.
- Fixed location matching: word-boundary state/city matching (was substring — 'la'
  matched 'Latin America'->Colombia, 'columbia' matched 'British Columbia', split
  'mexico'/'york' matched foreign cities). Full state names + curated city regex.
- Added 'engineer' title exclusion (Marvell optical 'CPO' false positive).
- 35 roles (fit 5x5 fintech, 4x14 AI, 3x6, 2x2, 1x8); 12 remote + 23 US-metro.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011C7n5R5VxejCKFAN8WmUQg
</commit_message>
<xml_diff>
--- a/research/fp-a-role-scan/product_leadership_roles.xlsx
+++ b/research/fp-a-role-scan/product_leadership_roles.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matches'!$A$2:$L$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matches'!$A$2:$L$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,7 +45,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +77,11 @@
         <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,6 +134,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -496,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -516,7 +524,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Product &amp; exec leadership • Director/Head/VP Product · CPO · COO · Founding PM • eligible with 12 yrs (min ≤12) • Remote-US / Dallas–Fort Worth / San Francisco • posted ≤60 days • Fit indexed on fintech/crypto/AI (5=fintech/crypto, 4=AI, 3=infra/SaaS, 2=other, 1=none)</t>
+          <t>Product &amp; exec leadership • Director/Head/VP Product · CPO · COO · Founding PM • eligible with 12 yrs (min ≤12) • any US location (remote or metro; filter by city) • posted ≤60 days • Fit: 5=fintech/crypto, 4=AI, 3=infra/SaaS, 2=other, 1=none</t>
         </is>
       </c>
     </row>
@@ -678,7 +686,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>San Francisco: San Francisco, California (in-office)</t>
+          <t>SF: San Francisco, California (in-office)</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -740,7 +748,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>San Francisco: San Francisco, California, United States</t>
+          <t>SF: San Francisco, California, United States</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -768,12 +776,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>GV</t>
+          <t>Lightspeed</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Tala</t>
+          <t>Flex</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -783,7 +791,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Director of Product</t>
+          <t>Director of Product, Payments Platform</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -793,20 +801,24 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>12+</t>
+          <t>7+</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Remote (US)</t>
+          <t>SF: San Francisco, California (in-office)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr"/>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>$248,000–$310,000</t>
+        </is>
+      </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
           <t>fintech / crypto / payments — priority domain</t>
@@ -826,12 +838,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Lightspeed</t>
+          <t>Founders Fund</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Flex</t>
+          <t>Rippling</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -841,34 +853,26 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Director of Product, Payments Platform</t>
+          <t>Senior Director of Product Management, Payroll</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>director</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>7+</t>
+          <t>n/s</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>San Francisco: San Francisco, California (in-office)</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>$248,000–$310,000</t>
-        </is>
-      </c>
+          <t>SF: San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
           <t>fintech / crypto / payments — priority domain</t>
@@ -881,19 +885,19 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Founders Fund</t>
+          <t>Felicis</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Rippling</t>
+          <t>Runlayer</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -903,12 +907,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Senior Director of Product Management, Payroll</t>
+          <t>Founding Product Manager, Control Plane</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -918,14 +922,22 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>San Francisco: San Francisco, CA</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>$135,000–$220,000</t>
+        </is>
+      </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>fintech / crypto / payments — priority domain</t>
+          <t>AI / ML — priority domain</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -957,7 +969,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Founding Product Manager, Control Plane</t>
+          <t>Founding Product Manager, Agents</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1004,12 +1016,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Felicis</t>
+          <t>IVP, Venrock</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Runlayer</t>
+          <t>Aledade</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1019,12 +1031,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Founding Product Manager, Agents</t>
+          <t>Director of Product Management (Internal AI Product Strategy &amp; Ops), Remote</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1039,14 +1051,10 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>$135,000–$220,000</t>
-        </is>
-      </c>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr">
         <is>
           <t>AI / ML — priority domain</t>
@@ -1066,12 +1074,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>IVP, Venrock</t>
+          <t>Spark Capital</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Aledade</t>
+          <t>Scale AI</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1081,7 +1089,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Director of Product Management (Internal AI Product Strategy &amp; Ops), Remote</t>
+          <t>Director of Product Management, Forward Deployed &amp; Strategy</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1091,12 +1099,12 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>n/s</t>
+          <t>10+</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Remote (US)</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1186,12 +1194,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Redpoint</t>
+          <t>Accel</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Codecov</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1201,7 +1209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Founding PM - Reporting &amp; Agentic Insights</t>
+          <t xml:space="preserve">Director of Product Management, AI Evals </t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1211,17 +1219,17 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>5+</t>
+          <t>8+</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Remote (US)</t>
+          <t>Mountain View, California, United States</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
@@ -1244,178 +1252,170 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Accel</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Director of Product Management, AI Evals </t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>8+</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Mountain View, California, United States</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Redpoint</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Founding PM - Reporting &amp; Agentic Insights</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>5+</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>Sequoia, a16z</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Instacart</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Public (CART)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Director of Product, Agentic Commerce</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>director</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>10+</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>$242,000–$307,000</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>AI / ML — priority domain</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>ContinuumCloud</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Director of Product Management</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>director</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>7+</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>$180,000–$285,000</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>data / infra / dev-tools / security SaaS</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>a16z</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Tanium</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Director of Product Management - Endpoint Management Partner Integrations</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>director</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>8+</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>DFW: DFW (hybrid)</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>$214,000–$328,000</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>data / infra / dev-tools / security SaaS</t>
-        </is>
-      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>apply ↗</t>
@@ -1423,9 +1423,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>iSpot.tv</t>
+          <t>CommerceIQ</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VP, Product Management </t>
+          <t>Director of Product Management - AI</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1455,211 +1455,1237 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>10+</t>
+          <t>6-12</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Remote (US)</t>
+          <t>Mountain View, California, United States</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr">
         <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Battery, GV, IVP</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Harness</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product Management, AI Evals</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>director</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>8+</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Mountain View, California (in-office)</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>$265,000–$280,000</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Lightspeed</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Normalyze</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>VP, Product Management, AI Data Security</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>vp</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Sunnyvale, California (in-office)</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>$200,000–$300,000</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Bessemer, GV, Lightspeed</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Nym Health</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product Management - Revenue Cycle AI</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>director</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>United States (in-office)</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>$180,000–$285,000</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Odyssey</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Head of Product</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>director</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Palo Alto, California (in-office)</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>$210,000–$300,000</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>AI / ML — priority domain</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Accel</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Celonis</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>VP, Product Management, Data Sources</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>n/s</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>New York, US, New York</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
           <t>data / infra / dev-tools / security SaaS</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>ContinuumCloud</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product Management</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>director</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>7+</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>$180,000–$285,000</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>data / infra / dev-tools / security SaaS</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>a16z</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Tanium</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product Management - Endpoint Management Partner Integrations</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>director</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>8+</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Bellevue, Washington (hybrid)</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>$214,000–$328,000</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>data / infra / dev-tools / security SaaS</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Insight Partners</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>iSpot.tv</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VP, Product Management </t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>data / infra / dev-tools / security SaaS</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Greylock</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Pepper</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Founding PM, Convenience Store</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>mid</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>5+</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>New York, New York (in-office)</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>$170,000–$250,000</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>data / infra / dev-tools / security SaaS</t>
+        </is>
+      </c>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>IVP</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Genlogs</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Director of Product- Shippers</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>n/s</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>data / infra / dev-tools / security SaaS</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Oak HC/FT, Sequoia</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Maven Clinic</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>VP of Product, Healthcare</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>vp</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>10+</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>$200,000–$300,000</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>other vertical (consumer / health / logistics / etc.)</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
-        <is>
-          <t>apply ↗</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>GV, IVP, Venrock, Lightspeed</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Aledade</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Director of Product Management (Salesforce), Remote</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>director</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>12+</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>Remote (US)</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>$180,000–$285,000</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>other vertical (consumer / health / logistics / etc.)</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Wonder</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Associate Director of Product, Blue Apron</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>director, manager</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>8+</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>United States (in-office)</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>$193,500–$203,000</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Wonder</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Associate Director of Product, Retention</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>director, manager</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>8+</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>United States (in-office)</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>$193,500–$203,000</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Spark Capital</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Formation Bio</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Senior Director or Vice President, Product</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>New York, NY; Boston MA</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Accel</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Fictiv</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Director of Product Management </t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Schaumburg, IL</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Oak HC/FT</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Pagaya</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Public (PGY)</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Head of Product, Personal Loans </t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Insight Partners</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Quince</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product, Growth</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Palo Alto, California, United States</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>8VC</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Hello Patient</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Head of Product</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>5+</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Austin, Texas</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>$200K – $250K • Offers Equity</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>apply ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Insight Partners</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Inspiren</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Director of Product Management, New Markets</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>7+</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>no clear domain overlap</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
         <is>
           <t>apply ↗</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L20"/>
+  <autoFilter ref="A2:L37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId2"/>
@@ -1679,6 +2705,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>